<commit_message>
Sprint 2: Actualizar esquema SQL, diccionario de datos, diagrama ER y plantilla de Jupyter Notebook
</commit_message>
<xml_diff>
--- a/MYOREHAB_Data_Dictionary.xlsx
+++ b/MYOREHAB_Data_Dictionary.xlsx
@@ -796,12 +796,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1152,6 +1152,141 @@
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>injuries_description</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>type of injuries</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Participant's sport</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>sport_type</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Type of sport practiced</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>sport_frequency</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Frequency of sport practiced in days in a week</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>temporal_mark</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD HH:MM:SS</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp of form submission or data entry</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>